<commit_message>
test(route-deviation-detection): fixture + asercje detectRouteDeviations (p5)
- test-data/sample-report.csv, test-data/sample-report.xlsx: rozszerzone o
  nowe kolumny (odwiedzony_klient/szerokosc/dlugosc) i 5 nowych wierszy
  pokrywających: poza planowaną trasą, nadmiarowy dystans, dwie reguły naraz,
  telefon pomijany przez regułę trasy, pierwsza wizyta dnia bez oceny dystansu
- scripts/verify-report-detection.mjs: rozszerzony o asercje
  detectRouteDeviations dla obu formatów (16/16 PASS); dodano lokalny resolve
  hook (node:module register, data: URL) dla aliasu @/* wymaganego przez
  realny import deviation-rules.ts -> geo.ts
</commit_message>
<xml_diff>
--- a/test-data/sample-report.xlsx
+++ b/test-data/sample-report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:J10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -421,6 +421,15 @@
       <c r="G1" t="str">
         <v>planowana_trasa</v>
       </c>
+      <c r="H1" t="str">
+        <v>odwiedzony_klient</v>
+      </c>
+      <c r="I1" t="str">
+        <v>szerokosc</v>
+      </c>
+      <c r="J1" t="str">
+        <v>dlugosc</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -444,6 +453,15 @@
       <c r="G2" t="str">
         <v>Klient A;Klient B</v>
       </c>
+      <c r="H2" t="str">
+        <v>Klient A</v>
+      </c>
+      <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -467,6 +485,15 @@
       <c r="G3" t="str">
         <v>Klient C</v>
       </c>
+      <c r="H3" t="str">
+        <v>Klient C</v>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -490,6 +517,15 @@
       <c r="G4" t="str">
         <v>Klient D;Klient E</v>
       </c>
+      <c r="H4" t="str">
+        <v>Klient D</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -513,10 +549,179 @@
       <c r="G5" t="str">
         <v>Klient F</v>
       </c>
+      <c r="H5" t="str">
+        <v>Klient F</v>
+      </c>
+      <c r="I5" t="str">
+        <v>52.3000</v>
+      </c>
+      <c r="J5" t="str">
+        <v>21.0000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>Ewa Testowa</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-09-03</v>
+      </c>
+      <c r="C6" t="str">
+        <v>TAK</v>
+      </c>
+      <c r="D6" t="str">
+        <v>wizyta</v>
+      </c>
+      <c r="E6" t="str">
+        <v>5</v>
+      </c>
+      <c r="F6" t="str">
+        <v>20</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Klient X;Klient Y</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Klient Z</v>
+      </c>
+      <c r="I6" t="str">
+        <v>52.2297</v>
+      </c>
+      <c r="J6" t="str">
+        <v>21.0122</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Marek Nowicki</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="C7" t="str">
+        <v>TAK</v>
+      </c>
+      <c r="D7" t="str">
+        <v>wizyta</v>
+      </c>
+      <c r="E7" t="str">
+        <v>5</v>
+      </c>
+      <c r="F7" t="str">
+        <v>15</v>
+      </c>
+      <c r="G7" t="str">
+        <v>Klient P;Klient Q</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Klient P</v>
+      </c>
+      <c r="I7" t="str">
+        <v>52.2297</v>
+      </c>
+      <c r="J7" t="str">
+        <v>21.0122</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Marek Nowicki</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-09-04</v>
+      </c>
+      <c r="C8" t="str">
+        <v>TAK</v>
+      </c>
+      <c r="D8" t="str">
+        <v>wizyta</v>
+      </c>
+      <c r="E8" t="str">
+        <v>15</v>
+      </c>
+      <c r="F8" t="str">
+        <v>10</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Klient P;Klient Q</v>
+      </c>
+      <c r="H8" t="str">
+        <v>Klient Q</v>
+      </c>
+      <c r="I8" t="str">
+        <v>52.2500</v>
+      </c>
+      <c r="J8" t="str">
+        <v>21.0300</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>Tomasz Kowalczyk</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-09-05</v>
+      </c>
+      <c r="C9" t="str">
+        <v>TAK</v>
+      </c>
+      <c r="D9" t="str">
+        <v>wizyta</v>
+      </c>
+      <c r="E9" t="str">
+        <v>5</v>
+      </c>
+      <c r="F9" t="str">
+        <v>15</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Klient R;Klient S</v>
+      </c>
+      <c r="H9" t="str">
+        <v>Klient R</v>
+      </c>
+      <c r="I9" t="str">
+        <v>52.2297</v>
+      </c>
+      <c r="J9" t="str">
+        <v>21.0122</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Tomasz Kowalczyk</v>
+      </c>
+      <c r="B10" t="str">
+        <v>2026-09-05</v>
+      </c>
+      <c r="C10" t="str">
+        <v>NIE</v>
+      </c>
+      <c r="D10" t="str">
+        <v>wizyta</v>
+      </c>
+      <c r="E10" t="str">
+        <v>15</v>
+      </c>
+      <c r="F10" t="str">
+        <v>10</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Klient R;Klient S</v>
+      </c>
+      <c r="H10" t="str">
+        <v>Klient S</v>
+      </c>
+      <c r="I10" t="str">
+        <v>52.2500</v>
+      </c>
+      <c r="J10" t="str">
+        <v>21.0300</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
test(phone-vs-visit-deviation-detection): fixture + asercje detectPhoneInsteadOfVisit (p3)
- test-data/sample-report.csv, test-data/sample-report.xlsx: rozszerzone o
  6 nowych wierszy (indeksy 9-14) pokrywających: wprost "telefon" (GPS
  niezależny), heurystyka z czasem=0, heurystyka z brakującym czasem (null
  jak zero), heurystyka z nierozpoznaną wartością typu, oraz dwa negatywy
  (GPS włączony, czas zbyt długi)
- scripts/verify-report-detection.mjs: rozszerzony o asercje
  detectPhoneInsteadOfVisit dla obu formatów (38/38 PASS), istniejące
  asercje missing_gps/route_deviation dla oryginalnych 9 wierszy nadal
  przechodzą niezmienione
</commit_message>
<xml_diff>
--- a/test-data/sample-report.xlsx
+++ b/test-data/sample-report.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J10"/>
+  <dimension ref="A1:J16"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -719,9 +719,201 @@
         <v>21.0300</v>
       </c>
     </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>Zofia Mazur</v>
+      </c>
+      <c r="B11" t="str">
+        <v>2026-09-06</v>
+      </c>
+      <c r="C11" t="str">
+        <v>TAK</v>
+      </c>
+      <c r="D11" t="str">
+        <v>telefon</v>
+      </c>
+      <c r="E11" t="str">
+        <v>0</v>
+      </c>
+      <c r="F11" t="str">
+        <v>30</v>
+      </c>
+      <c r="G11" t="str">
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <v>Klient T1</v>
+      </c>
+      <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>Robert Lis</v>
+      </c>
+      <c r="B12" t="str">
+        <v>2026-09-07</v>
+      </c>
+      <c r="C12" t="str">
+        <v>NIE</v>
+      </c>
+      <c r="D12" t="str">
+        <v/>
+      </c>
+      <c r="E12" t="str">
+        <v>0</v>
+      </c>
+      <c r="F12" t="str">
+        <v>0</v>
+      </c>
+      <c r="G12" t="str">
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <v>Klient T2</v>
+      </c>
+      <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>Lucyna Wrona</v>
+      </c>
+      <c r="B13" t="str">
+        <v>2026-09-08</v>
+      </c>
+      <c r="C13" t="str">
+        <v>NIE</v>
+      </c>
+      <c r="D13" t="str">
+        <v/>
+      </c>
+      <c r="E13" t="str">
+        <v>0</v>
+      </c>
+      <c r="F13" t="str">
+        <v/>
+      </c>
+      <c r="G13" t="str">
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <v>Klient T3</v>
+      </c>
+      <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>Marcin Duda</v>
+      </c>
+      <c r="B14" t="str">
+        <v>2026-09-09</v>
+      </c>
+      <c r="C14" t="str">
+        <v>NIE</v>
+      </c>
+      <c r="D14" t="str">
+        <v>spotkanie</v>
+      </c>
+      <c r="E14" t="str">
+        <v>0</v>
+      </c>
+      <c r="F14" t="str">
+        <v>0</v>
+      </c>
+      <c r="G14" t="str">
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <v>Klient T4</v>
+      </c>
+      <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Alicja Górecka</v>
+      </c>
+      <c r="B15" t="str">
+        <v>2026-09-10</v>
+      </c>
+      <c r="C15" t="str">
+        <v>TAK</v>
+      </c>
+      <c r="D15" t="str">
+        <v/>
+      </c>
+      <c r="E15" t="str">
+        <v>0</v>
+      </c>
+      <c r="F15" t="str">
+        <v>0</v>
+      </c>
+      <c r="G15" t="str">
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <v>Klient T5</v>
+      </c>
+      <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Katarzyna Woźniak</v>
+      </c>
+      <c r="B16" t="str">
+        <v>2026-09-11</v>
+      </c>
+      <c r="C16" t="str">
+        <v>NIE</v>
+      </c>
+      <c r="D16" t="str">
+        <v/>
+      </c>
+      <c r="E16" t="str">
+        <v>0</v>
+      </c>
+      <c r="F16" t="str">
+        <v>15</v>
+      </c>
+      <c r="G16" t="str">
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <v>Klient T6</v>
+      </c>
+      <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J10"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J16"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>